<commit_message>
Discriminativo anual das reduções da DBGG no cenário IPCA+0,37 p.p.
Apresenta, para cada ano de 2007 a 2026, a economia de juros da parcela
Selic (redução no ano), a diferença acumulada de estoque e a participação
no total, em Markdown, CSV e aba Discriminativo do Excel.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/dbgg_selic_ipca_2007_2026.xlsx
+++ b/output/dbgg_selic_ipca_2007_2026.xlsx
@@ -9,14 +9,15 @@
   <sheets>
     <sheet name="Mensal" sheetId="1" r:id="rId1"/>
     <sheet name="Anual" sheetId="2" r:id="rId2"/>
-    <sheet name="Notas" sheetId="3" r:id="rId3"/>
+    <sheet name="Discriminativo" sheetId="3" r:id="rId3"/>
+    <sheet name="Notas" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
   <si>
     <t>mes</t>
   </si>
@@ -88,6 +89,21 @@
   </si>
   <si>
     <t>economia_juros</t>
+  </si>
+  <si>
+    <t>reducao_ano</t>
+  </si>
+  <si>
+    <t>reducao_acumulada</t>
+  </si>
+  <si>
+    <t>variacao_delta_dbgg</t>
+  </si>
+  <si>
+    <t>participacao_pct</t>
+  </si>
+  <si>
+    <t>spread_selic_menos_cf</t>
   </si>
   <si>
     <t>campo</t>
@@ -14743,20 +14759,1395 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:21">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21">
+      <c r="A2">
+        <v>2007</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1">
+        <v>39417</v>
+      </c>
+      <c r="D2">
+        <v>4.45733043</v>
+      </c>
+      <c r="E2">
+        <v>4.82733043</v>
+      </c>
+      <c r="F2">
+        <v>11.84810729</v>
+      </c>
+      <c r="G2">
+        <v>63620.21865348</v>
+      </c>
+      <c r="H2">
+        <v>25947.29110706</v>
+      </c>
+      <c r="I2">
+        <v>37672.92754642</v>
+      </c>
+      <c r="J2">
+        <v>580232.78893847</v>
+      </c>
+      <c r="K2">
+        <v>542559.8613920501</v>
+      </c>
+      <c r="L2">
+        <v>1542851.83360594</v>
+      </c>
+      <c r="M2">
+        <v>1505178.90605952</v>
+      </c>
+      <c r="N2">
+        <v>37672.92754642</v>
+      </c>
+      <c r="O2">
+        <v>44.55</v>
+      </c>
+      <c r="P2">
+        <v>43.46219047</v>
+      </c>
+      <c r="Q2">
+        <v>37672.92754642</v>
+      </c>
+      <c r="R2">
+        <v>37672.92754642</v>
+      </c>
+      <c r="S2">
+        <v>37672.92754642</v>
+      </c>
+      <c r="T2">
+        <v>1.540701464328347</v>
+      </c>
+      <c r="U2">
+        <v>7.02077686</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3">
+        <v>2008</v>
+      </c>
+      <c r="B3">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1">
+        <v>39783</v>
+      </c>
+      <c r="D3">
+        <v>5.90231342</v>
+      </c>
+      <c r="E3">
+        <v>6.27231342</v>
+      </c>
+      <c r="F3">
+        <v>12.48098472</v>
+      </c>
+      <c r="G3">
+        <v>81636.834049</v>
+      </c>
+      <c r="H3">
+        <v>38490.38652033</v>
+      </c>
+      <c r="I3">
+        <v>43146.44752867</v>
+      </c>
+      <c r="J3">
+        <v>754748.9146576</v>
+      </c>
+      <c r="K3">
+        <v>673929.53958252</v>
+      </c>
+      <c r="L3">
+        <v>1740887.81455873</v>
+      </c>
+      <c r="M3">
+        <v>1660068.43948365</v>
+      </c>
+      <c r="N3">
+        <v>80819.37507508</v>
+      </c>
+      <c r="O3">
+        <v>37.57</v>
+      </c>
+      <c r="P3">
+        <v>35.82584171</v>
+      </c>
+      <c r="Q3">
+        <v>43146.44752867</v>
+      </c>
+      <c r="R3">
+        <v>80819.37507508</v>
+      </c>
+      <c r="S3">
+        <v>43146.44752865999</v>
+      </c>
+      <c r="T3">
+        <v>1.764550811881493</v>
+      </c>
+      <c r="U3">
+        <v>6.208671300000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21">
+      <c r="A4">
+        <v>2009</v>
+      </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1">
+        <v>40148</v>
+      </c>
+      <c r="D4">
+        <v>4.31202833</v>
+      </c>
+      <c r="E4">
+        <v>4.68202833</v>
+      </c>
+      <c r="F4">
+        <v>9.923897910000001</v>
+      </c>
+      <c r="G4">
+        <v>85054.06020592</v>
+      </c>
+      <c r="H4">
+        <v>36495.2220553</v>
+      </c>
+      <c r="I4">
+        <v>48558.83815062</v>
+      </c>
+      <c r="J4">
+        <v>931465.69848925</v>
+      </c>
+      <c r="K4">
+        <v>802087.48526355</v>
+      </c>
+      <c r="L4">
+        <v>1973423.68412051</v>
+      </c>
+      <c r="M4">
+        <v>1844045.47089481</v>
+      </c>
+      <c r="N4">
+        <v>129378.2132257</v>
+      </c>
+      <c r="O4">
+        <v>40.88</v>
+      </c>
+      <c r="P4">
+        <v>38.19989567</v>
+      </c>
+      <c r="Q4">
+        <v>48558.83815062</v>
+      </c>
+      <c r="R4">
+        <v>129378.2132257</v>
+      </c>
+      <c r="S4">
+        <v>48558.83815062001</v>
+      </c>
+      <c r="T4">
+        <v>1.985900165378918</v>
+      </c>
+      <c r="U4">
+        <v>5.241869580000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
+      <c r="A5">
+        <v>2010</v>
+      </c>
+      <c r="B5">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>40513</v>
+      </c>
+      <c r="D5">
+        <v>5.90906835</v>
+      </c>
+      <c r="E5">
+        <v>6.27906835</v>
+      </c>
+      <c r="F5">
+        <v>9.78245864</v>
+      </c>
+      <c r="G5">
+        <v>81872.25479137999</v>
+      </c>
+      <c r="H5">
+        <v>45143.0562304</v>
+      </c>
+      <c r="I5">
+        <v>36729.19856098</v>
+      </c>
+      <c r="J5">
+        <v>787279.4662747401</v>
+      </c>
+      <c r="K5">
+        <v>621172.0544880599</v>
+      </c>
+      <c r="L5">
+        <v>2011521.66204921</v>
+      </c>
+      <c r="M5">
+        <v>1845414.25026253</v>
+      </c>
+      <c r="N5">
+        <v>166107.41178668</v>
+      </c>
+      <c r="O5">
+        <v>37.98</v>
+      </c>
+      <c r="P5">
+        <v>34.84368801</v>
+      </c>
+      <c r="Q5">
+        <v>36729.19856098</v>
+      </c>
+      <c r="R5">
+        <v>166107.41178668</v>
+      </c>
+      <c r="S5">
+        <v>36729.19856097999</v>
+      </c>
+      <c r="T5">
+        <v>1.502105986766777</v>
+      </c>
+      <c r="U5">
+        <v>3.50339029</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
+      <c r="A6">
+        <v>2011</v>
+      </c>
+      <c r="B6">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
+        <v>40878</v>
+      </c>
+      <c r="D6">
+        <v>6.50310904</v>
+      </c>
+      <c r="E6">
+        <v>6.87310904</v>
+      </c>
+      <c r="F6">
+        <v>11.61582141</v>
+      </c>
+      <c r="G6">
+        <v>95780.34195118</v>
+      </c>
+      <c r="H6">
+        <v>45903.81212489</v>
+      </c>
+      <c r="I6">
+        <v>49876.52982629</v>
+      </c>
+      <c r="J6">
+        <v>869045.48143523</v>
+      </c>
+      <c r="K6">
+        <v>653061.53982226</v>
+      </c>
+      <c r="L6">
+        <v>2243603.71512325</v>
+      </c>
+      <c r="M6">
+        <v>2027619.77351028</v>
+      </c>
+      <c r="N6">
+        <v>215983.94161297</v>
+      </c>
+      <c r="O6">
+        <v>34.47</v>
+      </c>
+      <c r="P6">
+        <v>31.15169275</v>
+      </c>
+      <c r="Q6">
+        <v>49876.52982629</v>
+      </c>
+      <c r="R6">
+        <v>215983.94161297</v>
+      </c>
+      <c r="S6">
+        <v>49876.52982629</v>
+      </c>
+      <c r="T6">
+        <v>2.039789513153563</v>
+      </c>
+      <c r="U6">
+        <v>4.74271237</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21">
+      <c r="A7">
+        <v>2012</v>
+      </c>
+      <c r="B7">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>41244</v>
+      </c>
+      <c r="D7">
+        <v>5.838569</v>
+      </c>
+      <c r="E7">
+        <v>6.208569</v>
+      </c>
+      <c r="F7">
+        <v>8.482270939999999</v>
+      </c>
+      <c r="G7">
+        <v>77291.02458665</v>
+      </c>
+      <c r="H7">
+        <v>43330.49506903</v>
+      </c>
+      <c r="I7">
+        <v>33960.52951762</v>
+      </c>
+      <c r="J7">
+        <v>929446.57743525</v>
+      </c>
+      <c r="K7">
+        <v>679502.10630466</v>
+      </c>
+      <c r="L7">
+        <v>2583946.35443261</v>
+      </c>
+      <c r="M7">
+        <v>2334001.88330202</v>
+      </c>
+      <c r="N7">
+        <v>249944.47113059</v>
+      </c>
+      <c r="O7">
+        <v>32.19</v>
+      </c>
+      <c r="P7">
+        <v>29.07626952</v>
+      </c>
+      <c r="Q7">
+        <v>33960.52951762</v>
+      </c>
+      <c r="R7">
+        <v>249944.47113059</v>
+      </c>
+      <c r="S7">
+        <v>33960.52951762002</v>
+      </c>
+      <c r="T7">
+        <v>1.388876335471714</v>
+      </c>
+      <c r="U7">
+        <v>2.27370194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21">
+      <c r="A8">
+        <v>2013</v>
+      </c>
+      <c r="B8">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1">
+        <v>41609</v>
+      </c>
+      <c r="D8">
+        <v>5.91081808</v>
+      </c>
+      <c r="E8">
+        <v>6.28081808</v>
+      </c>
+      <c r="F8">
+        <v>8.21335618</v>
+      </c>
+      <c r="G8">
+        <v>85817.35720643</v>
+      </c>
+      <c r="H8">
+        <v>50120.78688669</v>
+      </c>
+      <c r="I8">
+        <v>35696.57031974</v>
+      </c>
+      <c r="J8">
+        <v>916591.9960370701</v>
+      </c>
+      <c r="K8">
+        <v>630950.95458675</v>
+      </c>
+      <c r="L8">
+        <v>2747996.70552741</v>
+      </c>
+      <c r="M8">
+        <v>2462355.66407709</v>
+      </c>
+      <c r="N8">
+        <v>285641.04145032</v>
+      </c>
+      <c r="O8">
+        <v>30.5</v>
+      </c>
+      <c r="P8">
+        <v>27.32967169</v>
+      </c>
+      <c r="Q8">
+        <v>35696.57031974</v>
+      </c>
+      <c r="R8">
+        <v>285641.04145032</v>
+      </c>
+      <c r="S8">
+        <v>35696.57031972997</v>
+      </c>
+      <c r="T8">
+        <v>1.459874815817163</v>
+      </c>
+      <c r="U8">
+        <v>1.932538099999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21">
+      <c r="A9">
+        <v>2014</v>
+      </c>
+      <c r="B9">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1">
+        <v>41974</v>
+      </c>
+      <c r="D9">
+        <v>6.4076166</v>
+      </c>
+      <c r="E9">
+        <v>6.7776166</v>
+      </c>
+      <c r="F9">
+        <v>10.91009207</v>
+      </c>
+      <c r="G9">
+        <v>107106.66927377</v>
+      </c>
+      <c r="H9">
+        <v>48636.87500753</v>
+      </c>
+      <c r="I9">
+        <v>58469.79426624</v>
+      </c>
+      <c r="J9">
+        <v>1226853.40074324</v>
+      </c>
+      <c r="K9">
+        <v>882742.56502668</v>
+      </c>
+      <c r="L9">
+        <v>3252448.54925185</v>
+      </c>
+      <c r="M9">
+        <v>2908337.71353529</v>
+      </c>
+      <c r="N9">
+        <v>344110.83571656</v>
+      </c>
+      <c r="O9">
+        <v>32.59</v>
+      </c>
+      <c r="P9">
+        <v>29.14196017</v>
+      </c>
+      <c r="Q9">
+        <v>58469.79426624</v>
+      </c>
+      <c r="R9">
+        <v>344110.83571656</v>
+      </c>
+      <c r="S9">
+        <v>58469.79426624003</v>
+      </c>
+      <c r="T9">
+        <v>2.391226366307011</v>
+      </c>
+      <c r="U9">
+        <v>4.132475469999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21">
+      <c r="A10">
+        <v>2015</v>
+      </c>
+      <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1">
+        <v>42339</v>
+      </c>
+      <c r="D10">
+        <v>10.673498</v>
+      </c>
+      <c r="E10">
+        <v>11.043498</v>
+      </c>
+      <c r="F10">
+        <v>13.2857836</v>
+      </c>
+      <c r="G10">
+        <v>170372.33365925</v>
+      </c>
+      <c r="H10">
+        <v>103963.76526972</v>
+      </c>
+      <c r="I10">
+        <v>66408.56838953</v>
+      </c>
+      <c r="J10">
+        <v>1539457.14413662</v>
+      </c>
+      <c r="K10">
+        <v>1128937.74003052</v>
+      </c>
+      <c r="L10">
+        <v>3927523.06280055</v>
+      </c>
+      <c r="M10">
+        <v>3517003.65869445</v>
+      </c>
+      <c r="N10">
+        <v>410519.4041061</v>
+      </c>
+      <c r="O10">
+        <v>35.64</v>
+      </c>
+      <c r="P10">
+        <v>31.91477386</v>
+      </c>
+      <c r="Q10">
+        <v>66408.56838953</v>
+      </c>
+      <c r="R10">
+        <v>410519.4041061</v>
+      </c>
+      <c r="S10">
+        <v>66408.56838953996</v>
+      </c>
+      <c r="T10">
+        <v>2.715896672368404</v>
+      </c>
+      <c r="U10">
+        <v>2.242285600000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21">
+      <c r="A11">
+        <v>2016</v>
+      </c>
+      <c r="B11">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1">
+        <v>42705</v>
+      </c>
+      <c r="D11">
+        <v>6.28805505</v>
+      </c>
+      <c r="E11">
+        <v>6.65805505</v>
+      </c>
+      <c r="F11">
+        <v>14.02838763</v>
+      </c>
+      <c r="G11">
+        <v>232251.36223635</v>
+      </c>
+      <c r="H11">
+        <v>83131.83372747</v>
+      </c>
+      <c r="I11">
+        <v>149119.52850888</v>
+      </c>
+      <c r="J11">
+        <v>1918752.38231828</v>
+      </c>
+      <c r="K11">
+        <v>1359113.44970331</v>
+      </c>
+      <c r="L11">
+        <v>4378486.39497225</v>
+      </c>
+      <c r="M11">
+        <v>3818847.46235728</v>
+      </c>
+      <c r="N11">
+        <v>559638.93261497</v>
+      </c>
+      <c r="O11">
+        <v>46.14</v>
+      </c>
+      <c r="P11">
+        <v>40.24258751</v>
+      </c>
+      <c r="Q11">
+        <v>149119.52850888</v>
+      </c>
+      <c r="R11">
+        <v>559638.93261497</v>
+      </c>
+      <c r="S11">
+        <v>149119.52850887</v>
+      </c>
+      <c r="T11">
+        <v>6.098508687717231</v>
+      </c>
+      <c r="U11">
+        <v>7.370332579999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21">
+      <c r="A12">
+        <v>2017</v>
+      </c>
+      <c r="B12">
+        <v>12</v>
+      </c>
+      <c r="C12" s="1">
+        <v>43070</v>
+      </c>
+      <c r="D12">
+        <v>2.94734991</v>
+      </c>
+      <c r="E12">
+        <v>3.31734991</v>
+      </c>
+      <c r="F12">
+        <v>9.955642320000001</v>
+      </c>
+      <c r="G12">
+        <v>195121.73108859</v>
+      </c>
+      <c r="H12">
+        <v>47538.47378515</v>
+      </c>
+      <c r="I12">
+        <v>147583.25730344</v>
+      </c>
+      <c r="J12">
+        <v>2177104.98508228</v>
+      </c>
+      <c r="K12">
+        <v>1469882.79516387</v>
+      </c>
+      <c r="L12">
+        <v>4854678.58647316</v>
+      </c>
+      <c r="M12">
+        <v>4147456.39655475</v>
+      </c>
+      <c r="N12">
+        <v>707222.18991841</v>
+      </c>
+      <c r="O12">
+        <v>51.37</v>
+      </c>
+      <c r="P12">
+        <v>43.88649656</v>
+      </c>
+      <c r="Q12">
+        <v>147583.25730344</v>
+      </c>
+      <c r="R12">
+        <v>707222.18991841</v>
+      </c>
+      <c r="S12">
+        <v>147583.25730344</v>
+      </c>
+      <c r="T12">
+        <v>6.035680140800872</v>
+      </c>
+      <c r="U12">
+        <v>6.638292410000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21">
+      <c r="A13">
+        <v>2018</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1">
+        <v>43435</v>
+      </c>
+      <c r="D13">
+        <v>3.74548212</v>
+      </c>
+      <c r="E13">
+        <v>4.11548212</v>
+      </c>
+      <c r="F13">
+        <v>6.4215212</v>
+      </c>
+      <c r="G13">
+        <v>140704.40894162</v>
+      </c>
+      <c r="H13">
+        <v>62937.56874871</v>
+      </c>
+      <c r="I13">
+        <v>77766.84019290999</v>
+      </c>
+      <c r="J13">
+        <v>2509463.41400522</v>
+      </c>
+      <c r="K13">
+        <v>1724474.3838939</v>
+      </c>
+      <c r="L13">
+        <v>5271982.25856809</v>
+      </c>
+      <c r="M13">
+        <v>4486993.22845677</v>
+      </c>
+      <c r="N13">
+        <v>784989.03011131</v>
+      </c>
+      <c r="O13">
+        <v>52.77</v>
+      </c>
+      <c r="P13">
+        <v>44.91263837</v>
+      </c>
+      <c r="Q13">
+        <v>77766.84019290999</v>
+      </c>
+      <c r="R13">
+        <v>784989.03011131</v>
+      </c>
+      <c r="S13">
+        <v>77766.84019289992</v>
+      </c>
+      <c r="T13">
+        <v>3.180413425895033</v>
+      </c>
+      <c r="U13">
+        <v>2.30603908</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21">
+      <c r="A14">
+        <v>2019</v>
+      </c>
+      <c r="B14">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1">
+        <v>43800</v>
+      </c>
+      <c r="D14">
+        <v>4.30603998</v>
+      </c>
+      <c r="E14">
+        <v>4.67603998</v>
+      </c>
+      <c r="F14">
+        <v>5.94594036</v>
+      </c>
+      <c r="G14">
+        <v>153195.22615653</v>
+      </c>
+      <c r="H14">
+        <v>85239.42788156</v>
+      </c>
+      <c r="I14">
+        <v>67955.79827497</v>
+      </c>
+      <c r="J14">
+        <v>2644895.86473309</v>
+      </c>
+      <c r="K14">
+        <v>1791951.0363468</v>
+      </c>
+      <c r="L14">
+        <v>5500104.15654906</v>
+      </c>
+      <c r="M14">
+        <v>4647159.32816277</v>
+      </c>
+      <c r="N14">
+        <v>852944.82838629</v>
+      </c>
+      <c r="O14">
+        <v>54.7</v>
+      </c>
+      <c r="P14">
+        <v>46.21723662</v>
+      </c>
+      <c r="Q14">
+        <v>67955.79827497</v>
+      </c>
+      <c r="R14">
+        <v>852944.82838629</v>
+      </c>
+      <c r="S14">
+        <v>67955.79827498004</v>
+      </c>
+      <c r="T14">
+        <v>2.779173394019852</v>
+      </c>
+      <c r="U14">
+        <v>1.26990038</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21">
+      <c r="A15">
+        <v>2020</v>
+      </c>
+      <c r="B15">
+        <v>12</v>
+      </c>
+      <c r="C15" s="1">
+        <v>44166</v>
+      </c>
+      <c r="D15">
+        <v>4.5173415</v>
+      </c>
+      <c r="E15">
+        <v>4.8873415</v>
+      </c>
+      <c r="F15">
+        <v>2.75381578</v>
+      </c>
+      <c r="G15">
+        <v>79806.42598997999</v>
+      </c>
+      <c r="H15">
+        <v>104494.00141297</v>
+      </c>
+      <c r="I15">
+        <v>-24687.57542299</v>
+      </c>
+      <c r="J15">
+        <v>3046581.63859695</v>
+      </c>
+      <c r="K15">
+        <v>2218324.38563365</v>
+      </c>
+      <c r="L15">
+        <v>6615755.2038528</v>
+      </c>
+      <c r="M15">
+        <v>5787497.9508895</v>
+      </c>
+      <c r="N15">
+        <v>828257.2529633</v>
+      </c>
+      <c r="O15">
+        <v>61.37</v>
+      </c>
+      <c r="P15">
+        <v>53.68680344</v>
+      </c>
+      <c r="Q15">
+        <v>-24687.57542299</v>
+      </c>
+      <c r="R15">
+        <v>828257.2529633</v>
+      </c>
+      <c r="S15">
+        <v>-24687.57542299002</v>
+      </c>
+      <c r="T15">
+        <v>-1.009642363419981</v>
+      </c>
+      <c r="U15">
+        <v>-2.13352572</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21">
+      <c r="A16">
+        <v>2021</v>
+      </c>
+      <c r="B16">
+        <v>12</v>
+      </c>
+      <c r="C16" s="1">
+        <v>44531</v>
+      </c>
+      <c r="D16">
+        <v>10.06105489</v>
+      </c>
+      <c r="E16">
+        <v>10.43105489</v>
+      </c>
+      <c r="F16">
+        <v>4.43568776</v>
+      </c>
+      <c r="G16">
+        <v>138565.90883077</v>
+      </c>
+      <c r="H16">
+        <v>239001.16719482</v>
+      </c>
+      <c r="I16">
+        <v>-100435.25836405</v>
+      </c>
+      <c r="J16">
+        <v>3117259.54614057</v>
+      </c>
+      <c r="K16">
+        <v>2389437.55154132</v>
+      </c>
+      <c r="L16">
+        <v>6966925.20075086</v>
+      </c>
+      <c r="M16">
+        <v>6239103.20615161</v>
+      </c>
+      <c r="N16">
+        <v>727821.99459925</v>
+      </c>
+      <c r="O16">
+        <v>55.11</v>
+      </c>
+      <c r="P16">
+        <v>49.35275861</v>
+      </c>
+      <c r="Q16">
+        <v>-100435.25836405</v>
+      </c>
+      <c r="R16">
+        <v>727821.99459925</v>
+      </c>
+      <c r="S16">
+        <v>-100435.25836405</v>
+      </c>
+      <c r="T16">
+        <v>-4.107478757551257</v>
+      </c>
+      <c r="U16">
+        <v>-5.99536713</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21">
+      <c r="A17">
+        <v>2022</v>
+      </c>
+      <c r="B17">
+        <v>12</v>
+      </c>
+      <c r="C17" s="1">
+        <v>44896</v>
+      </c>
+      <c r="D17">
+        <v>5.78484196</v>
+      </c>
+      <c r="E17">
+        <v>6.15484196</v>
+      </c>
+      <c r="F17">
+        <v>12.38048663</v>
+      </c>
+      <c r="G17">
+        <v>396376.86557541</v>
+      </c>
+      <c r="H17">
+        <v>151290.7526861</v>
+      </c>
+      <c r="I17">
+        <v>245086.11288931</v>
+      </c>
+      <c r="J17">
+        <v>3269588.27164342</v>
+      </c>
+      <c r="K17">
+        <v>2296680.16415486</v>
+      </c>
+      <c r="L17">
+        <v>7224882.23036494</v>
+      </c>
+      <c r="M17">
+        <v>6251974.12287638</v>
+      </c>
+      <c r="N17">
+        <v>972908.10748856</v>
+      </c>
+      <c r="O17">
+        <v>56.13</v>
+      </c>
+      <c r="P17">
+        <v>48.57149173</v>
+      </c>
+      <c r="Q17">
+        <v>245086.11288931</v>
+      </c>
+      <c r="R17">
+        <v>972908.10748856</v>
+      </c>
+      <c r="S17">
+        <v>245086.11288931</v>
+      </c>
+      <c r="T17">
+        <v>10.02323306437558</v>
+      </c>
+      <c r="U17">
+        <v>6.22564467</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21">
+      <c r="A18">
+        <v>2023</v>
+      </c>
+      <c r="B18">
+        <v>12</v>
+      </c>
+      <c r="C18" s="1">
+        <v>45261</v>
+      </c>
+      <c r="D18">
+        <v>4.62111393</v>
+      </c>
+      <c r="E18">
+        <v>4.99111393</v>
+      </c>
+      <c r="F18">
+        <v>13.02823091</v>
+      </c>
+      <c r="G18">
+        <v>464903.10176633</v>
+      </c>
+      <c r="H18">
+        <v>127868.30816077</v>
+      </c>
+      <c r="I18">
+        <v>337034.79360556</v>
+      </c>
+      <c r="J18">
+        <v>3892563.64661376</v>
+      </c>
+      <c r="K18">
+        <v>2582620.74551964</v>
+      </c>
+      <c r="L18">
+        <v>8079270.02452043</v>
+      </c>
+      <c r="M18">
+        <v>6769327.12342631</v>
+      </c>
+      <c r="N18">
+        <v>1309942.90109412</v>
+      </c>
+      <c r="O18">
+        <v>60.43</v>
+      </c>
+      <c r="P18">
+        <v>50.63210375</v>
+      </c>
+      <c r="Q18">
+        <v>337034.79360556</v>
+      </c>
+      <c r="R18">
+        <v>1309942.90109412</v>
+      </c>
+      <c r="S18">
+        <v>337034.79360556</v>
+      </c>
+      <c r="T18">
+        <v>13.78363811513857</v>
+      </c>
+      <c r="U18">
+        <v>8.03711698</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21">
+      <c r="A19">
+        <v>2024</v>
+      </c>
+      <c r="B19">
+        <v>12</v>
+      </c>
+      <c r="C19" s="1">
+        <v>45627</v>
+      </c>
+      <c r="D19">
+        <v>4.83129579</v>
+      </c>
+      <c r="E19">
+        <v>5.20129579</v>
+      </c>
+      <c r="F19">
+        <v>10.88812643</v>
+      </c>
+      <c r="G19">
+        <v>483616.92215309</v>
+      </c>
+      <c r="H19">
+        <v>160414.28076729</v>
+      </c>
+      <c r="I19">
+        <v>323202.6413858</v>
+      </c>
+      <c r="J19">
+        <v>4757243.88275394</v>
+      </c>
+      <c r="K19">
+        <v>3124098.34027402</v>
+      </c>
+      <c r="L19">
+        <v>8984236.59444961</v>
+      </c>
+      <c r="M19">
+        <v>7351091.05196968</v>
+      </c>
+      <c r="N19">
+        <v>1633145.54247992</v>
+      </c>
+      <c r="O19">
+        <v>61.3</v>
+      </c>
+      <c r="P19">
+        <v>50.15694731</v>
+      </c>
+      <c r="Q19">
+        <v>323202.6413858</v>
+      </c>
+      <c r="R19">
+        <v>1633145.54247992</v>
+      </c>
+      <c r="S19">
+        <v>323202.6413858</v>
+      </c>
+      <c r="T19">
+        <v>13.21794761621099</v>
+      </c>
+      <c r="U19">
+        <v>5.68683064</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21">
+      <c r="A20">
+        <v>2025</v>
+      </c>
+      <c r="B20">
+        <v>12</v>
+      </c>
+      <c r="C20" s="1">
+        <v>45992</v>
+      </c>
+      <c r="D20">
+        <v>4.2643849</v>
+      </c>
+      <c r="E20">
+        <v>4.6343849</v>
+      </c>
+      <c r="F20">
+        <v>14.33275639</v>
+      </c>
+      <c r="G20">
+        <v>697542.74516402</v>
+      </c>
+      <c r="H20">
+        <v>147852.53259141</v>
+      </c>
+      <c r="I20">
+        <v>549690.21257261</v>
+      </c>
+      <c r="J20">
+        <v>5286916.60437279</v>
+      </c>
+      <c r="K20">
+        <v>3104080.84932025</v>
+      </c>
+      <c r="L20">
+        <v>10017919.13888715</v>
+      </c>
+      <c r="M20">
+        <v>7835083.38383461</v>
+      </c>
+      <c r="N20">
+        <v>2182835.75505254</v>
+      </c>
+      <c r="O20">
+        <v>65.23999999999999</v>
+      </c>
+      <c r="P20">
+        <v>51.02465221</v>
+      </c>
+      <c r="Q20">
+        <v>549690.21257261</v>
+      </c>
+      <c r="R20">
+        <v>2182835.75505254</v>
+      </c>
+      <c r="S20">
+        <v>549690.21257262</v>
+      </c>
+      <c r="T20">
+        <v>22.4805601952233</v>
+      </c>
+      <c r="U20">
+        <v>9.69837149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21">
+      <c r="A21">
+        <v>2026</v>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+      <c r="C21" s="1">
+        <v>46174</v>
+      </c>
+      <c r="D21">
+        <v>3.36449142</v>
+      </c>
+      <c r="E21">
+        <v>3.54949142</v>
+      </c>
+      <c r="F21">
+        <v>6.83686668</v>
+      </c>
+      <c r="G21">
+        <v>379312.39305751</v>
+      </c>
+      <c r="H21">
+        <v>116967.92217686</v>
+      </c>
+      <c r="I21">
+        <v>262344.47088065</v>
+      </c>
+      <c r="J21">
+        <v>5861746.95005535</v>
+      </c>
+      <c r="K21">
+        <v>3416566.72412216</v>
+      </c>
+      <c r="L21">
+        <v>10809475.19418525</v>
+      </c>
+      <c r="M21">
+        <v>8364294.96825206</v>
+      </c>
+      <c r="N21">
+        <v>2445180.22593319</v>
+      </c>
+      <c r="O21">
+        <v>68.48</v>
+      </c>
+      <c r="P21">
+        <v>52.98933659</v>
+      </c>
+      <c r="Q21">
+        <v>262344.47088065</v>
+      </c>
+      <c r="R21">
+        <v>2445180.22593319</v>
+      </c>
+      <c r="S21">
+        <v>262344.47088065</v>
+      </c>
+      <c r="T21">
+        <v>10.72904435011642</v>
+      </c>
+      <c r="U21">
+        <v>3.28737526</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B2">
         <v>0.37</v>
@@ -14764,34 +16155,34 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>